<commit_message>
[add] UnlockConditionData 테스트용 5연승 해금조건 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/UnlockConditionData.xlsx
+++ b/JsonConverter/ExcelFiles/UnlockConditionData.xlsx
@@ -19,7 +19,61 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+  <x:si>
+    <x:t>5연승</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cond_streak_5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cond_win_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WinStreak</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TargetId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>item_aaa</x:t>
+  </x:si>
+  <x:si>
+    <x:t>아이템 aaa보유</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Type</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HasItem</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Count</x:t>
+  </x:si>
+  <x:si>
+    <x:t>None</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>전체 1승</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
   <x:si>
     <x:t>3연승</x:t>
   </x:si>
@@ -27,58 +81,10 @@
     <x:t>cond_streak_3</x:t>
   </x:si>
   <x:si>
+    <x:t>cond_item_aaa</x:t>
+  </x:si>
+  <x:si>
     <x:t>TotalWinCount</x:t>
-  </x:si>
-  <x:si>
-    <x:t>cond_item_aaa</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Count</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HasItem</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Type</x:t>
-  </x:si>
-  <x:si>
-    <x:t>전체 1승</x:t>
-  </x:si>
-  <x:si>
-    <x:t>None</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WinStreak</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>cond_win_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>아이템 aaa보유</x:t>
-  </x:si>
-  <x:si>
-    <x:t>item_aaa</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TargetId</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -865,99 +871,111 @@
   <x:sheetData>
     <x:row r="1" spans="1:1" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5" s="7" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="2" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E3" s="7" t="s">
         <x:v>4</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C3" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="D3" s="7" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E3" s="7" t="s">
-        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>15</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>2</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C4" s="3">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D4" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E4" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F4" s="4"/>
     </x:row>
     <x:row r="5" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
-        <x:v>1</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C5" s="3">
         <x:v>3</x:v>
       </x:c>
       <x:c r="D5" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E5" s="1" t="s">
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5" ht="15.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
-        <x:v>3</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>7</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C6" s="5">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A7" s="5"/>
-      <x:c r="B7" s="5"/>
-      <x:c r="C7" s="5"/>
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="A7" s="5" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C7" s="5">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" spans="1:3" ht="15.75" customHeight="1">
       <x:c r="A8" s="5"/>

</xml_diff>